<commit_message>
Atualiza dashboard e scripts de otimização
</commit_message>
<xml_diff>
--- a/data/loads.xlsx
+++ b/data/loads.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inesctecpt-my.sharepoint.com/personal/diana_f_rodrigues_inesctec_pt/Documents/Documents/pypsa/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inesctecpt-my.sharepoint.com/personal/diana_f_rodrigues_inesctec_pt/Documents/Documents/pypsa/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="11_F25DC773A252ABDACC10484139184E125BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98CCA374-7966-47D7-BBDE-5653BCF98C5C}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="11_F25DC773A252ABDACC10484139184E125BDE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8909DCF4-9313-4729-8F7A-ECBE9899FF2B}"/>
   <bookViews>
-    <workbookView xWindow="25017" yWindow="-118" windowWidth="25370" windowHeight="13667" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="759" yWindow="759" windowWidth="18851" windowHeight="9766" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="12">
   <si>
     <t>name</t>
   </si>
@@ -33,22 +33,34 @@
     <t>bus</t>
   </si>
   <si>
-    <t>Ventilation</t>
-  </si>
-  <si>
-    <t>Pumps</t>
-  </si>
-  <si>
-    <t>Lighting</t>
-  </si>
-  <si>
-    <t>Equipment</t>
-  </si>
-  <si>
-    <t>Cooling</t>
-  </si>
-  <si>
     <t>electricity</t>
+  </si>
+  <si>
+    <t>carrier</t>
+  </si>
+  <si>
+    <t>equipment_main</t>
+  </si>
+  <si>
+    <t>lighting_main</t>
+  </si>
+  <si>
+    <t>ventilation</t>
+  </si>
+  <si>
+    <t>pumping</t>
+  </si>
+  <si>
+    <t>cooling</t>
+  </si>
+  <si>
+    <t>equipment</t>
+  </si>
+  <si>
+    <t>lighting</t>
+  </si>
+  <si>
+    <t>category</t>
   </si>
 </sst>
 </file>
@@ -366,59 +378,95 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>